<commit_message>
Refine error processing and update reports
Removed commented-out code and improved error categorization logic in processamento_erros.py, including broader handling of invalid characters in error messages. Updated multiple Excel reports and added a new PDF report for 07.07.2025.
</commit_message>
<xml_diff>
--- a/Integration Quality/EMPRESAS/Relatorio - ZUPPER VIAGENS.xlsx
+++ b/Integration Quality/EMPRESAS/Relatorio - ZUPPER VIAGENS.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ5"/>
+  <dimension ref="A1:AQ8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -695,10 +695,10 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
-        <v>22507625</v>
+        <v>22510237</v>
       </c>
       <c r="B2" s="5" t="n">
-        <v>23340279</v>
+        <v>23342278</v>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
@@ -706,34 +706,34 @@
         </is>
       </c>
       <c r="D2" s="6" t="n">
-        <v>45841.92925925926</v>
+        <v>45842.51754629629</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>45841.92967592592</v>
+        <v>45842.52206018518</v>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>JEANHF</t>
+          <t>TFN85Y</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>EBOOKING</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Dalila Lisboa</t>
+          <t>JULIANA SOUZA</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
@@ -743,14 +743,14 @@
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>Zupper</t>
+          <t>Ananda Maia Fernandes</t>
         </is>
       </c>
       <c r="M2" s="6" t="n">
-        <v>45841.92847222222</v>
+        <v>45842.51736111111</v>
       </c>
       <c r="N2" s="5" t="n">
-        <v>6767181</v>
+        <v>6642873</v>
       </c>
       <c r="O2" s="5" t="inlineStr">
         <is>
@@ -764,12 +764,12 @@
       </c>
       <c r="Q2" s="5" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="R2" s="5" t="inlineStr">
         <is>
-          <t>Cartão convênio</t>
+          <t>TKT</t>
         </is>
       </c>
       <c r="S2" s="5" t="inlineStr">
@@ -789,7 +789,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>Dalila Maria de Fatima Lisboa</t>
+          <t>Juliana dos Santos Souza</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -799,11 +799,11 @@
       </c>
       <c r="X2" s="5" t="inlineStr">
         <is>
-          <t>Latam Airlines Brasil</t>
+          <t>Azul Linhas Aereas</t>
         </is>
       </c>
       <c r="Y2" s="5" t="n">
-        <v>2239718681</v>
+        <v>3023342315</v>
       </c>
       <c r="Z2" s="5" t="inlineStr">
         <is>
@@ -816,10 +816,10 @@
         </is>
       </c>
       <c r="AB2" s="5" t="n">
-        <v>138.32</v>
+        <v>0</v>
       </c>
       <c r="AC2" s="5" t="n">
-        <v>30.95</v>
+        <v>0</v>
       </c>
       <c r="AD2" s="5" t="n">
         <v>0</v>
@@ -834,7 +834,7 @@
         <v>0</v>
       </c>
       <c r="AH2" s="5" t="n">
-        <v>25.55</v>
+        <v>0</v>
       </c>
       <c r="AI2" s="5" t="inlineStr">
         <is>
@@ -884,10 +884,10 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>22505120</v>
+        <v>22521118</v>
       </c>
       <c r="B3" s="5" t="n">
-        <v>23337831</v>
+        <v>23350522</v>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
@@ -895,10 +895,10 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>45841.66396990741</v>
+        <v>45845.04261574074</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>45841.66504629629</v>
+        <v>45845.04484953704</v>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
@@ -912,7 +912,7 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>VWSCGN</t>
+          <t>DYIMIT</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>Gisela Gibson Freitas</t>
+          <t>Wellinna Araujo</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
@@ -936,10 +936,10 @@
         </is>
       </c>
       <c r="M3" s="6" t="n">
-        <v>45841.66319444445</v>
+        <v>45845.04097222222</v>
       </c>
       <c r="N3" s="5" t="n">
-        <v>6766386</v>
+        <v>6769933</v>
       </c>
       <c r="O3" s="5" t="inlineStr">
         <is>
@@ -978,7 +978,7 @@
       </c>
       <c r="V3" s="5" t="inlineStr">
         <is>
-          <t>Gisela Gibson de Freitas</t>
+          <t>Wellinna Gleicy Lobato Araujo</t>
         </is>
       </c>
       <c r="W3" s="5" t="inlineStr">
@@ -988,11 +988,11 @@
       </c>
       <c r="X3" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y3" s="5" t="n">
-        <v>5226286672</v>
+        <v>2240093151</v>
       </c>
       <c r="Z3" s="5" t="inlineStr">
         <is>
@@ -1005,10 +1005,10 @@
         </is>
       </c>
       <c r="AB3" s="5" t="n">
-        <v>885.39</v>
+        <v>614.6900000000001</v>
       </c>
       <c r="AC3" s="5" t="n">
-        <v>51.92</v>
+        <v>51.07</v>
       </c>
       <c r="AD3" s="5" t="n">
         <v>0</v>
@@ -1023,7 +1023,7 @@
         <v>0</v>
       </c>
       <c r="AH3" s="5" t="n">
-        <v>159.36</v>
+        <v>78.84</v>
       </c>
       <c r="AI3" s="5" t="inlineStr">
         <is>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="AJ3" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data transação 03/07/2025</t>
+          <t>Pnr já existente. A duplicidade de rloc é permitida apenas 6 meses após o último pnr emitido</t>
         </is>
       </c>
       <c r="AK3" s="5" t="inlineStr">
@@ -1042,17 +1042,17 @@
       </c>
       <c r="AL3" s="5" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>Duplicidade de RLOC</t>
         </is>
       </c>
       <c r="AM3" s="5" t="inlineStr">
         <is>
-          <t>Análise Benner</t>
+          <t>Campo RLOC</t>
         </is>
       </c>
       <c r="AN3" s="5" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Duplicidade de Contabilização</t>
         </is>
       </c>
       <c r="AO3" s="5" t="inlineStr">
@@ -1073,21 +1073,21 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
-        <v>22505120</v>
+        <v>22521609</v>
       </c>
       <c r="B4" s="5" t="n">
-        <v>23337832</v>
+        <v>23350788</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>ACC02</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>45841.66396990741</v>
+        <v>45845.20449074074</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>45841.66504629629</v>
+        <v>45845.20670138889</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>VWSCGN</t>
+          <t>SUSQIX</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Marcelo Gibson Freitas Souza</t>
+          <t>BRUNA Leda</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -1125,10 +1125,10 @@
         </is>
       </c>
       <c r="M4" s="6" t="n">
-        <v>45841.66319444445</v>
+        <v>45845.20277777778</v>
       </c>
       <c r="N4" s="5" t="n">
-        <v>6766386</v>
+        <v>6770003</v>
       </c>
       <c r="O4" s="5" t="inlineStr">
         <is>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>Gisela Gibson de Freitas</t>
+          <t>Bruna Mayara Fernandes Leda</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1177,11 +1177,11 @@
       </c>
       <c r="X4" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y4" s="5" t="n">
-        <v>2800792721</v>
+        <v>2240099058</v>
       </c>
       <c r="Z4" s="5" t="inlineStr">
         <is>
@@ -1194,10 +1194,10 @@
         </is>
       </c>
       <c r="AB4" s="5" t="n">
-        <v>885.39</v>
+        <v>523.92</v>
       </c>
       <c r="AC4" s="5" t="n">
-        <v>51.92</v>
+        <v>111.69</v>
       </c>
       <c r="AD4" s="5" t="n">
         <v>0</v>
@@ -1212,7 +1212,7 @@
         <v>0</v>
       </c>
       <c r="AH4" s="5" t="n">
-        <v>0</v>
+        <v>67.48999999999999</v>
       </c>
       <c r="AI4" s="5" t="inlineStr">
         <is>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="AJ4" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data transação 03/07/2025</t>
+          <t>Pnr já existente. A duplicidade de rloc é permitida apenas 6 meses após o último pnr emitido</t>
         </is>
       </c>
       <c r="AK4" s="5" t="inlineStr">
@@ -1231,17 +1231,17 @@
       </c>
       <c r="AL4" s="5" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>Duplicidade de RLOC</t>
         </is>
       </c>
       <c r="AM4" s="5" t="inlineStr">
         <is>
-          <t>Análise Benner</t>
+          <t>Campo RLOC</t>
         </is>
       </c>
       <c r="AN4" s="5" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Duplicidade de Contabilização</t>
         </is>
       </c>
       <c r="AO4" s="5" t="inlineStr">
@@ -1262,21 +1262,21 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>22505120</v>
+        <v>22514438</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>23337833</v>
+        <v>23346135</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>ACC03</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>45841.66396990741</v>
+        <v>45843.04265046296</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>45841.66504629629</v>
+        <v>45843.04458333334</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
@@ -1290,7 +1290,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>VWSCGN</t>
+          <t>WQLBOC</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>Luana Gibson Freitas Souza</t>
+          <t>Mirtes Vieira</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
@@ -1314,10 +1314,10 @@
         </is>
       </c>
       <c r="M5" s="6" t="n">
-        <v>45841.66319444445</v>
+        <v>45843.04097222222</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>6766386</v>
+        <v>6768388</v>
       </c>
       <c r="O5" s="5" t="inlineStr">
         <is>
@@ -1356,7 +1356,7 @@
       </c>
       <c r="V5" s="5" t="inlineStr">
         <is>
-          <t>Gisela Gibson de Freitas</t>
+          <t>Marina Jacauna Vieira</t>
         </is>
       </c>
       <c r="W5" s="5" t="inlineStr">
@@ -1366,11 +1366,11 @@
       </c>
       <c r="X5" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y5" s="5" t="n">
-        <v>5990216094</v>
+        <v>2239886983</v>
       </c>
       <c r="Z5" s="5" t="inlineStr">
         <is>
@@ -1383,10 +1383,10 @@
         </is>
       </c>
       <c r="AB5" s="5" t="n">
-        <v>885.39</v>
+        <v>832.72</v>
       </c>
       <c r="AC5" s="5" t="n">
-        <v>51.92</v>
+        <v>46.36</v>
       </c>
       <c r="AD5" s="5" t="n">
         <v>0</v>
@@ -1401,7 +1401,7 @@
         <v>0</v>
       </c>
       <c r="AH5" s="5" t="n">
-        <v>0</v>
+        <v>212.18</v>
       </c>
       <c r="AI5" s="5" t="inlineStr">
         <is>
@@ -1410,7 +1410,7 @@
       </c>
       <c r="AJ5" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data transação 03/07/2025</t>
+          <t>Pnr já existente. A duplicidade de rloc é permitida apenas 6 meses após o último pnr emitido</t>
         </is>
       </c>
       <c r="AK5" s="5" t="inlineStr">
@@ -1420,17 +1420,17 @@
       </c>
       <c r="AL5" s="5" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>Duplicidade de RLOC</t>
         </is>
       </c>
       <c r="AM5" s="5" t="inlineStr">
         <is>
-          <t>Análise Benner</t>
+          <t>Campo RLOC</t>
         </is>
       </c>
       <c r="AN5" s="5" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Duplicidade de Contabilização</t>
         </is>
       </c>
       <c r="AO5" s="5" t="inlineStr">
@@ -1444,6 +1444,573 @@
         </is>
       </c>
       <c r="AQ5" s="5" t="inlineStr">
+        <is>
+          <t>Operações - ZUPPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>22514438</v>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>23346136</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>ACC02</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>45843.04265046296</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>45843.04458333334</v>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>0 a 02 dias</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>0 a 02 dias</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>WQLBOC</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>EBOOKING</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Mirelle Vieira</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="M6" s="6" t="n">
+        <v>45843.04097222222</v>
+      </c>
+      <c r="N6" s="5" t="n">
+        <v>6768388</v>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P6" s="5" t="inlineStr">
+        <is>
+          <t>OFF LINE</t>
+        </is>
+      </c>
+      <c r="Q6" s="5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="R6" s="5" t="inlineStr">
+        <is>
+          <t>Cartão convênio</t>
+        </is>
+      </c>
+      <c r="S6" s="5" t="inlineStr">
+        <is>
+          <t>Aéreo</t>
+        </is>
+      </c>
+      <c r="T6" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U6" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Zupper</t>
+        </is>
+      </c>
+      <c r="V6" s="5" t="inlineStr">
+        <is>
+          <t>Marina Jacauna Vieira</t>
+        </is>
+      </c>
+      <c r="W6" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X6" s="5" t="inlineStr">
+        <is>
+          <t>Latam Airlines Brasil</t>
+        </is>
+      </c>
+      <c r="Y6" s="5" t="n">
+        <v>2239886984</v>
+      </c>
+      <c r="Z6" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AA6" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB6" s="5" t="n">
+        <v>832.72</v>
+      </c>
+      <c r="AC6" s="5" t="n">
+        <v>46.36</v>
+      </c>
+      <c r="AD6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI6" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ6" s="5" t="inlineStr">
+        <is>
+          <t>Pnr já existente. A duplicidade de rloc é permitida apenas 6 meses após o último pnr emitido</t>
+        </is>
+      </c>
+      <c r="AK6" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AL6" s="5" t="inlineStr">
+        <is>
+          <t>Duplicidade de RLOC</t>
+        </is>
+      </c>
+      <c r="AM6" s="5" t="inlineStr">
+        <is>
+          <t>Campo RLOC</t>
+        </is>
+      </c>
+      <c r="AN6" s="5" t="inlineStr">
+        <is>
+          <t>Duplicidade de Contabilização</t>
+        </is>
+      </c>
+      <c r="AO6" s="5" t="inlineStr">
+        <is>
+          <t>Qualidade dos dados</t>
+        </is>
+      </c>
+      <c r="AP6" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER VIAGENS</t>
+        </is>
+      </c>
+      <c r="AQ6" s="5" t="inlineStr">
+        <is>
+          <t>Operações - ZUPPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>22515553</v>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>23346784</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>ACC01</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>45843.48627314815</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>45843.48797453703</v>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>0 a 02 dias</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>0 a 02 dias</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>CBRH94</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>EBOOKING</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Felipe Bernacchi</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>45843.48541666667</v>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>6768128</v>
+      </c>
+      <c r="O7" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P7" s="5" t="inlineStr">
+        <is>
+          <t>OFF LINE</t>
+        </is>
+      </c>
+      <c r="Q7" s="5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="R7" s="5" t="inlineStr">
+        <is>
+          <t>Cartão convênio</t>
+        </is>
+      </c>
+      <c r="S7" s="5" t="inlineStr">
+        <is>
+          <t>Aéreo</t>
+        </is>
+      </c>
+      <c r="T7" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U7" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Zupper</t>
+        </is>
+      </c>
+      <c r="V7" s="5" t="inlineStr">
+        <is>
+          <t>Felipe Bernacchi</t>
+        </is>
+      </c>
+      <c r="W7" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X7" s="5" t="inlineStr">
+        <is>
+          <t>Taag</t>
+        </is>
+      </c>
+      <c r="Y7" s="5" t="n">
+        <v>2971441399</v>
+      </c>
+      <c r="Z7" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AA7" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB7" s="5" t="n">
+        <v>3241.63</v>
+      </c>
+      <c r="AC7" s="5" t="n">
+        <v>347.94</v>
+      </c>
+      <c r="AD7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI7" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ7" s="5" t="inlineStr">
+        <is>
+          <t>'*' is not a valid integer value</t>
+        </is>
+      </c>
+      <c r="AK7" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AL7" s="5" t="inlineStr">
+        <is>
+          <t>Caractere inválido</t>
+        </is>
+      </c>
+      <c r="AM7" s="5" t="inlineStr">
+        <is>
+          <t>Caractere invalido em campo gerencial</t>
+        </is>
+      </c>
+      <c r="AN7" s="5" t="inlineStr">
+        <is>
+          <t>Dados Gerenciais</t>
+        </is>
+      </c>
+      <c r="AO7" s="5" t="inlineStr">
+        <is>
+          <t>Qualidade dos dados</t>
+        </is>
+      </c>
+      <c r="AP7" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER VIAGENS</t>
+        </is>
+      </c>
+      <c r="AQ7" s="5" t="inlineStr">
+        <is>
+          <t>Operações - ZUPPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>22515553</v>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>23346785</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>ACC02</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>45843.48627314815</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>45843.48797453703</v>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>0 a 02 dias</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>0 a 02 dias</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>CBRH94</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>EBOOKING</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Grazielly Oliveira</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="M8" s="6" t="n">
+        <v>45843.48541666667</v>
+      </c>
+      <c r="N8" s="5" t="n">
+        <v>6768128</v>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P8" s="5" t="inlineStr">
+        <is>
+          <t>OFF LINE</t>
+        </is>
+      </c>
+      <c r="Q8" s="5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>Cartão convênio</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>Aéreo</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Zupper</t>
+        </is>
+      </c>
+      <c r="V8" s="5" t="inlineStr">
+        <is>
+          <t>Felipe Bernacchi</t>
+        </is>
+      </c>
+      <c r="W8" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X8" s="5" t="inlineStr">
+        <is>
+          <t>Taag</t>
+        </is>
+      </c>
+      <c r="Y8" s="5" t="n">
+        <v>2971441401</v>
+      </c>
+      <c r="Z8" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AA8" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB8" s="5" t="n">
+        <v>3241.63</v>
+      </c>
+      <c r="AC8" s="5" t="n">
+        <v>347.94</v>
+      </c>
+      <c r="AD8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI8" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ8" s="5" t="inlineStr">
+        <is>
+          <t>'*' is not a valid integer value</t>
+        </is>
+      </c>
+      <c r="AK8" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AL8" s="5" t="inlineStr">
+        <is>
+          <t>Caractere inválido</t>
+        </is>
+      </c>
+      <c r="AM8" s="5" t="inlineStr">
+        <is>
+          <t>Caractere invalido em campo gerencial</t>
+        </is>
+      </c>
+      <c r="AN8" s="5" t="inlineStr">
+        <is>
+          <t>Dados Gerenciais</t>
+        </is>
+      </c>
+      <c r="AO8" s="5" t="inlineStr">
+        <is>
+          <t>Qualidade dos dados</t>
+        </is>
+      </c>
+      <c r="AP8" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER VIAGENS</t>
+        </is>
+      </c>
+      <c r="AQ8" s="5" t="inlineStr">
         <is>
           <t>Operações - ZUPPER</t>
         </is>

</xml_diff>